<commit_message>
Update reference files (fills with patternType="none" removed)
</commit_message>
<xml_diff>
--- a/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
+++ b/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
@@ -427,21 +427,12 @@
   <x:dxfs count="3">
     <x:dxf>
       <x:numFmt numFmtId="15" formatCode="d-MMM-yy"/>
-      <x:fill>
-        <x:patternFill patternType="none"/>
-      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:numFmt numFmtId="164" formatCode="$ #,##0"/>
-      <x:fill>
-        <x:patternFill patternType="none"/>
-      </x:fill>
     </x:dxf>
     <x:dxf>
       <x:numFmt numFmtId="165" formatCode="0.00"/>
-      <x:fill>
-        <x:patternFill patternType="none"/>
-      </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>

</xml_diff>

<commit_message>
Copies of tables should have RelId default to null
</commit_message>
<xml_diff>
--- a/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
+++ b/ClosedXML_Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
@@ -1131,9 +1131,9 @@
     <x:firstFooter/>
   </x:headerFooter>
   <x:tableParts count="3">
-    <x:tablePart r:id="rId5"/>
-    <x:tablePart r:id="rId7"/>
-    <x:tablePart r:id="rId8"/>
+    <x:tablePart r:id="rId12"/>
+    <x:tablePart r:id="rId13"/>
+    <x:tablePart r:id="rId14"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>